<commit_message>
Done completely with Demoblaze
</commit_message>
<xml_diff>
--- a/DatadrivenTest_Framework/src/test/resources/dataset.xlsx
+++ b/DatadrivenTest_Framework/src/test/resources/dataset.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{D932F164-CEC6-4C6C-8301-7E92350E7F57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{BB7DC382-2110-4D09-AA7E-94C4509A0D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -381,7 +381,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B3">
@@ -401,6 +401,7 @@
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" xr:uid="{EFB45C06-51B0-4E97-887F-791F356ECC58}"/>
     <hyperlink ref="A4" r:id="rId2" xr:uid="{9CB9794E-F600-40BF-A4D3-DE161C22EA50}"/>
+    <hyperlink ref="A3" r:id="rId3" display="Admin@5" xr:uid="{EC60F241-454A-43EE-9D47-4E683E049960}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>